<commit_message>
docs: wave-2 review + response (rooftop bypass, s14 transfers, steam floor, funnel decision); analysis: transfer KPIs, wave-3/open selectors, storage export
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
(cherry picked from commit 3d3b7bbac4870597758e76b2d500575efb15801d)
</commit_message>
<xml_diff>
--- a/docs/proposals/NA_scenario_plan_2026-09-18_v4.xlsx
+++ b/docs/proposals/NA_scenario_plan_2026-09-18_v4.xlsx
@@ -8,23 +8,24 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Wave2_changes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overview" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Feasibility" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Model baseline" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Existing sensitivities" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Open questions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Wave3_changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wave2_changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Overview" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Feasibility" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Model baseline" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Existing sensitivities" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Open questions" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overview'!$A$1:$N$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Assumptions'!$A$1:$L$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Feasibility'!$A$1:$F$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources'!$A$1:$F$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Model baseline'!$A$1:$F$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Existing sensitivities'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Open questions'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Overview'!$A$1:$N$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Assumptions'!$A$1:$L$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Feasibility'!$A$1:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sources'!$A$1:$F$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Model baseline'!$A$1:$F$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Existing sensitivities'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Open questions'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -624,7 +625,531 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Why it matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Basis: v6 freeze - DECIDED (2026-09-22).</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Wave 1 = one variant per scenario (14 runs, serial, ~1 h each) - implemented; stretch/secondary variants (1B/1C, 2B/2C/2D, 3B/3C, 4B, 5B/5C, 6A/6B/6D, 7A/7B/7D, 8B/8C, 9A/9B, 10A/10B, 11B/11C, 12B/12C, 13B/13C, 14B/14C) on request.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Run budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Fusion: bull case implemented (base case available as a variant); NA location share (100 %) and site split are assumptions.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Confirm if a different NA share is wanted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Canada DC: scenario numbers used although below the FEL base (user rule); results will show a demand cut vs base - to be read as "announcement-consistent".</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>3 / 12</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>DC paths use the external-anchored numbers (not FEL presets).</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Consistency with published FEL numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Flat electrolysis load (2A); flexible electrolysers (2D) not built.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Capacity results at 333 TWh flat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>6C combined case implemented; the LNG-only / macro-only split (6A/6B) on request.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>10C dials implemented (10/20 % relocation).</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Overlap with FEL base industry growth unknown (FEL team) - adders applied on top.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Possible double counting in s13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>CO2 price 30/60/90 USD/t; nuclear ITC not added (unknown whether LCOE v1.4 nets it); CCS retrofit technology only in 14C (not built).</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Exogenous rip-and-replace capex report (11C) not built.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>4C run without the orbital-compute reduction (tailwind reading); the space_dc trio remains the displacement analysis.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>1 / 6</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Oil-shock/EV coupling only in 6D (not run).</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>RES supply-side brake included in 5A (rep funnel without the x1.30 widening).</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Wave 3 (2026-09-24/25): base-data fixes from the wave-2 review + funnel-released twins</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>change</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>reason (review finding)</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>run labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Rooftop PV build-rate cap: subset RooftopPV (P_PV_Rooftop_Commercial), GroupTotalAnnualMaxNewCap RooftopPV x USA = 7 GW/yr 2026-30 -&gt; 10 GW/yr 2040 (EIA small-scale additions 6.4 GW 2022, STEO 44 -&gt; 55 GW 2023-24; growth assumed). New base RegularParameters_NorthAmerica_v6f</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>N1: rooftop had no pipeline minimum and no build-rate limit and bypassed the utility-PV funnel at ~31 GW/yr (4x the US record); it drove the solar response in s05/s10/s12/s14 and the s06 pre-build (N2)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_base_49_2015_v6f</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Gas steam: guardrail minimum clamped to the residual fleet (31 rows: Canada, NY, SPP, ERCOT, NE)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>N4: flat post-2035 minimum forced ~12 GW of new steam units at a placeholder capex</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_base_49_2015_v6f</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>rerun on v6f; definitions otherwise unchanged</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>identical setup across the set</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_sNN_&lt;name&gt;_49_2015_v6_v3 (s03/s06 _v4, s14 _v5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>s10</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>coastal availability cut ramps -1 pp/yr 2030-34 (was a -5 pp step in 2030)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>N6: the step removed 10 % of the residual CCGT energy in one year (+97 TWh OCGT in 2030)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s10_climate_49_2015_v6_v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>twins</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>funnel-released twin of every scenario except s05: parent overlays + gas guardrail minimum = residual capacity from 2031 (announced projects through 2030 kept), build-rate caps unchanged; base NOT released (user decision)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>review item 2 / funnel debate: forced 366 GW of new CCGT+OCGT contradict s14/s07/s12; s05 already releases from 2027</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_sNN_&lt;name&gt;_open_49_2015_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>s14</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>no change; results now report ITC (193 bEUR disc.), 45Q (24) and CO2 payments (322) -&gt; resource cost +166 bEUR</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr"/>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>results</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>docs/proposals/scenario_plan_2026-09-18/RESULTS_wave3_2026-09-25.md; response docs/proposals/scenario_results/REVIEW_RESPONSE_wave2_2026-09-24.md</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -825,7 +1350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1908,7 +2433,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8659,7 +9184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9584,7 +10109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14087,7 +14612,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14822,7 +15347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14971,327 +15496,4 @@
   <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Why it matters</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Basis: v6 freeze - DECIDED (2026-09-22).</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Wave 1 = one variant per scenario (14 runs, serial, ~1 h each) - implemented; stretch/secondary variants (1B/1C, 2B/2C/2D, 3B/3C, 4B, 5B/5C, 6A/6B/6D, 7A/7B/7D, 8B/8C, 9A/9B, 10A/10B, 11B/11C, 12B/12C, 13B/13C, 14B/14C) on request.</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Run budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Fusion: bull case implemented (base case available as a variant); NA location share (100 %) and site split are assumptions.</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Confirm if a different NA share is wanted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Canada DC: scenario numbers used although below the FEL base (user rule); results will show a demand cut vs base - to be read as "announcement-consistent".</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>3 / 12</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>DC paths use the external-anchored numbers (not FEL presets).</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Consistency with published FEL numbers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Flat electrolysis load (2A); flexible electrolysers (2D) not built.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Capacity results at 333 TWh flat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>6C combined case implemented; the LNG-only / macro-only split (6A/6B) on request.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>10C dials implemented (10/20 % relocation).</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Overlap with FEL base industry growth unknown (FEL team) - adders applied on top.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Possible double counting in s13.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>CO2 price 30/60/90 USD/t; nuclear ITC not added (unknown whether LCOE v1.4 nets it); CCS retrofit technology only in 14C (not built).</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Exogenous rip-and-replace capex report (11C) not built.</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>4C run without the orbital-compute reduction (tailwind reading); the space_dc trio remains the displacement analysis.</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>1 / 6</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Oil-shock/EV coupling only in 6D (not run).</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>RES supply-side brake included in 5A (rep funnel without the x1.30 widening).</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D15"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: wave-4 results (hub-feedback set on base v6f, Hormuz variants, peaking diagnostic) + mapping, storage tables, plan sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
(cherry picked from commit 1f7df590df5bd34122eac416f4cff535bf1e8f48)
</commit_message>
<xml_diff>
--- a/docs/proposals/NA_scenario_plan_2026-09-18_v4.xlsx
+++ b/docs/proposals/NA_scenario_plan_2026-09-18_v4.xlsx
@@ -8,24 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Wave3_changes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wave2_changes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Overview" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Assumptions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Feasibility" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Model baseline" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Existing sensitivities" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Open questions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Wave4_changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Wave3_changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Wave2_changes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Overview" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Feasibility" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Model baseline" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Existing sensitivities" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Open questions" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Overview'!$A$1:$N$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Assumptions'!$A$1:$L$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Feasibility'!$A$1:$F$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sources'!$A$1:$F$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Model baseline'!$A$1:$F$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Existing sensitivities'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Open questions'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Overview'!$A$1:$N$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Assumptions'!$A$1:$L$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Feasibility'!$A$1:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources'!$A$1:$F$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Model baseline'!$A$1:$F$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Existing sensitivities'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Open questions'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -631,6 +632,157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Sensitivity (v6 set)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>dc_high</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>DC US 2035/2040 = 2188/3585 TWh; funnel max raised with ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>dc_low</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>DC US 2035/2040 = 805/874 TWh; gas min floor 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>recession</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>GDP-recession FEL demand: DC 1048/1563, General -1..2 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>btm_lag</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>DC 1526/2163 (BTM lag -&gt; more grid load)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>economic</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>funnel widened after 2030 (min x0.75, max x1.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>grid_high/grid_low</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>IC growth 2x budget / capped 0.75 %/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>bess_optimistic/pessimistic</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Li-ion cost x0.4 by 2040 + 7 h / min blend x0.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>nuclear_announced (+ccgtrelax)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>+19.1 GW announced nuclear (large+SMR) by 2035 on top of the corridor, CCGT min relaxed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>space_dc / disruptive / spacex</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>orbital compute REMOVES 5 / 13 / 27 % of US DC load by 2040 (1724/1585/1353 TWh)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>gas (NorthAmerica_gas)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>explicit gas supply, pipelines, LNG exports, storage, deliverability caps; endogenous regional gas prices</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -954,19 +1106,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Wave 3 (2026-09-24/25): base-data fixes from the wave-2 review + funnel-released twins</t>
+          <t>Wave 4 (2026-10-02): NA Hub market-intelligence feedback applied to the set on the unchanged base v6f (July freeze)</t>
         </is>
       </c>
     </row>
@@ -983,12 +1135,12 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>reason (review finding)</t>
+          <t>reason / source</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>run labels</t>
+          <t>run label</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1152,12 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Rooftop PV build-rate cap: subset RooftopPV (P_PV_Rooftop_Commercial), GroupTotalAnnualMaxNewCap RooftopPV x USA = 7 GW/yr 2026-30 -&gt; 10 GW/yr 2040 (EIA small-scale additions 6.4 GW 2022, STEO 44 -&gt; 55 GW 2023-24; growth assumed). New base RegularParameters_NorthAmerica_v6f</t>
+          <t>unchanged (v6f). Nuclear restart/uprate wave and named 45Q CCS projects recorded as v7 baseline items (stay inside s14)</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>N1: rooftop had no pipeline minimum and no build-rate limit and bypassed the utility-PV funnel at ~31 GW/yr (4x the US record); it drove the solar response in s05/s10/s12/s14 and the s06 pre-build (N2)</t>
+          <t>user decision: frozen truth, bugfixes only</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -1017,132 +1169,440 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>s01</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Gas steam: guardrail minimum clamped to the residual fleet (31 rows: Canada, NY, SPP, ERCOT, NE)</t>
+          <t>re-sized: +20 TWh BEV load in 2030 (share 23 % vs 10 %), AEO2026-shaped after (+49 TWh 2040); Canada base</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>N4: flat post-2035 minimum forced ~12 GW of new steam units at a placeholder capex</t>
+          <t>hub: full snap-back = 16-21 TWh by 2030; hybrids add no load</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>fel2026_base_49_2015_v6f</t>
+          <t>fel2026_s01_ev_49_2015_v6_v4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>s02</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>rerun on v6f; definitions otherwise unchanged</t>
+          <t>dropped as a run (wave-3 result citable)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>identical setup across the set</t>
+          <t>hub: electrolytic H2 below the FEL flat case; activity is CCS-backed (#14)</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>fel2026_sNN_&lt;name&gt;_49_2015_v6_v3 (s03/s06 _v4, s14 _v5)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>s10</t>
+          <t>s03</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>coastal availability cut ramps -1 pp/yr 2030-34 (was a -5 pp step in 2030)</t>
+          <t>unchanged; Hormuz variant added</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>N6: the step removed 10 % of the residual CCGT energy in one year (+97 TWh OCGT in 2030)</t>
+          <t>hub: High/Strong; contracted floor / supply ceiling band in the write-up</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>fel2026_s10_climate_49_2015_v6_v3</t>
+          <t>fel2026_s03_compute_49_2015_v6_v4 (wave 3), ..._hormuz_49_2015_v6</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>twins</t>
+          <t>s04</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>funnel-released twin of every scenario except s05: parent overlays + gas guardrail minimum = residual capacity from 2031 (announced projects through 2030 kept), build-rate caps unchanged; base NOT released (user decision)</t>
+          <t>dropped as a run; Starbase LA/TX point loads inside s13</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>review item 2 / funnel debate: forced 366 GW of new CCGT+OCGT contradict s14/s07/s12; s05 already releases from 2027</t>
+          <t>hub: Gulf-Coast named-account play, not a national load driver</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>fel2026_sNN_&lt;name&gt;_open_49_2015_v6</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>s14</t>
+          <t>s05</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>no change; results now report ITC (193 bEUR disc.), 45Q (24) and CO2 payments (322) -&gt; resource cost +166 bEUR</t>
+          <t>DC increment delayed 2 yr (ERCOT/NY 3) and cut to the credible tranche (55 %, ERCOT 66 %); gas release 2027, RES rule, cap window unchanged</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>N3</t>
+          <t>hub: delay not destruction; Texas audit + permit halt, NY moratorium; user chose delay + cut</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fel2026_s05_brakes_49_2015_v6_v4 (+ _hormuz)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr"/>
-      <c r="B9" s="9" t="inlineStr"/>
-      <c r="C9" s="9" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>s06</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>fuel-price channel only (Henry-Hub uplift 2026-30 via allFuels_v6_s06); capex/WACC uplift, IC cap, recession demand dropped</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>hub: live condition; capex plans rose, not frozen; cross-scenario sensitivity</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s06_hormuz_49_2015_v6_v5</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
+          <t>s07a</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>new split: iron-air from 2027 + optimistic Li-ion; gas minimum = residual from 2031</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>hub: LDES erodes peakers 2027-31</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s07a_ldes_49_2015_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>s07b</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>new split: fusion ramp 2034-40 + SMR 5,500-&gt;3,600 USD/kW; gas minimum = residual from 2031</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>hub: fusion/SMR post-2032 erode baseload</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s07b_fusion_49_2015_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>s08</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>unchanged (wave-3 run); Canada document pending (DRM-protected)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>hub: Alberta BYOP = base input (inside the CER gas path)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s08_canada_49_2015_v6_v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>s09</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>dropped as a run</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>hub: immaterial; water = siting constraint</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>s10</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>relocation 0 % (2035) / 5 % (2040) instead of 10/20 %; cooling, derate ramp, coastal IC cost kept</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>hub: relocation lags beyond the MEP27 horizon; resilience capex</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s10_climate_49_2015_v6_v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>s11</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>+ Section 232 transformer tariff (IC expansion cost x1.2 x1.15)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>hub proposal D (tariffs = cost and lead time)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s11_feoc_49_2015_v6_v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>s12</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>speculative tranche only: DC = 2026 + 55 % of the FEL increment to 2030 (ERCOT 66 %), flat 2031-32, FEL growth after; gas minimum = residual from 2031</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>hub: 101 of 182 GW credible (Currence/Jefferies); capex digestion 2031-32</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s12_overbuild_49_2015_v6_v4 (+ _hormuz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>s13</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>30 GW by 2035 (236 TWh at 90 % LF, flat after) on the wave-3 regional pattern + Starbase LA 2 GW (SERC), Starbase TX + chip plant 2 GW (ERCOT), Permian O&amp;G 1.6 GW (SPP); point-load sizes assumed</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>hub: elevate toward base; TransAlta ~30 GW; SPS peak +32 %</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s13_reindustrial_49_2015_v6_v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>s14</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>gas minimum = residual from 2031; CO2 price, ITC, 45Q, CCS cap, announced nuclear, state caps unchanged</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>funnel contradicts a 90 USD/t policy world (user decision)</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s14_decarb_49_2015_v6_v6 (+ _hormuz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>s15</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>new: grid-connected DC increment delayed 1 yr (large-load tariffs); IC growth = v6 grid_low path; BYOG 40 % of the DC increment reported as a metric (no model footprint)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>hub proposal A (#15 affordability / cost allocation)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s15_afford_49_2015_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>s16</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>new: v6 grid_high interconnector path (IC budget 2x by 2040); gas funnel as base</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>hub proposal F (transmission supercycle)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s16_gridhigh_49_2015_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>s17</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>diagnostic pair instead of a scenario: base with the peaking constraint on (slack 1.0) and with 10 % of DC peak curtailable (0.975)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>hub proposal G; no active firm-capacity constraint in the NA runs (set_peaking_slack = 0)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_base_peaking_49_2015_v6f, ..._flexdc_...</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Hormuz</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>fuel uplift as a variant of s03, s05, s12, s14 (allFuels swap, no new workbooks)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>hub: apply as baseline sensitivity across scenarios; base itself not changed</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_sNN_&lt;name&gt;_hormuz_49_2015_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr"/>
+      <c r="B23" s="9" t="inlineStr"/>
+      <c r="C23" s="9" t="inlineStr"/>
+      <c r="D23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
           <t>results</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>docs/proposals/scenario_plan_2026-09-18/RESULTS_wave3_2026-09-25.md; response docs/proposals/scenario_results/REVIEW_RESPONSE_wave2_2026-09-24.md</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>docs/proposals/scenario_plan_2026-09-18/RESULTS_wave4_2026-10-02.md; s14_summary_wave4.csv; scenario_mapping.csv updated</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr"/>
+      <c r="D24" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1161,35 +1621,35 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Wave 2 (2026-09-23/24): all 14 scenarios and the base rerun on one identical setup after the wave-1 review</t>
+          <t>Wave 3 (2026-09-24/25): base-data fixes from the wave-2 review + funnel-released twins</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>scenario</t>
+          <t>item</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>change vs plan v3 / wave 1</t>
+          <t>change</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>reason (review item)</t>
+          <t>reason (review finding)</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>wave-2 run label</t>
+          <t>run labels</t>
         </is>
       </c>
     </row>
@@ -1201,105 +1661,105 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Biogas co-firing mode (mode 2, Gas_Bio) disabled for all gas plants in the BASE data (OutputActivityRatio Power = 0); new base RegularParameters_NorthAmerica_v6e</t>
+          <t>Rooftop PV build-rate cap: subset RooftopPV (P_PV_Rooftop_Commercial), GroupTotalAnnualMaxNewCap RooftopPV x USA = 7 GW/yr 2026-30 -&gt; 10 GW/yr 2040 (EIA small-scale additions 6.4 GW 2022, STEO 44 -&gt; 55 GW 2023-24; growth assumed). New base RegularParameters_NorthAmerica_v6f</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Review #1: mode 2 = unlimited zero-CO2 gas in the power-only data, understated 2030 CO2 by ~600 Mt in every v6 run</t>
+          <t>N1: rooftop had no pipeline minimum and no build-rate limit and bypassed the utility-PV funnel at ~31 GW/yr (4x the US record); it drove the solar response in s05/s10/s12/s14 and the s06 pre-build (N2)</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>fel2026_base_49_2015_v6e</t>
+          <t>fel2026_base_49_2015_v6f</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>base</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>rerun on the fixed base data; definitions otherwise unchanged</t>
+          <t>Gas steam: guardrail minimum clamped to the residual fleet (31 rows: Canada, NY, SPP, ERCOT, NE)</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>identical setup across the set</t>
+          <t>N4: flat post-2035 minimum forced ~12 GW of new steam units at a placeholder capex</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>fel2026_sNN_&lt;name&gt;_49_2015_v6_v2</t>
+          <t>fel2026_base_49_2015_v6f</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>s03</t>
+          <t>all</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>crypto adder = growth above today's load: 0 TWh 2026, +10 TWh 2030, +20 TWh 2035/40 (was on from 2025)</t>
+          <t>rerun on v6f; definitions otherwise unchanged</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Review #3: crypto double-counted (already in the FEL base load)</t>
+          <t>identical setup across the set</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>fel2026_s03_compute_49_2015_v6_v2</t>
+          <t>fel2026_sNN_&lt;name&gt;_49_2015_v6_v3 (s03/s06 _v4, s14 _v5)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>s05</t>
+          <t>s10</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>separate GasEngines window cap (min(base,1) GW/yr 2027-31) next to the GasPlants cap min(base,10) GW/yr 2027-31; engines NOT in GasPlants (base GasPlants 6/9/10 GW caps would collide)</t>
+          <t>coastal availability cut ramps -1 pp/yr 2030-34 (was a -5 pp step in 2030)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Review #12: 2028 gas additions exceeded the cap via engines outside the subset</t>
+          <t>N6: the step removed 10 % of the residual CCGT energy in one year (+97 TWh OCGT in 2030)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>fel2026_s05_brakes_49_2015_v6_v2</t>
+          <t>fel2026_s10_climate_49_2015_v6_v3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>s06</t>
+          <t>twins</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>capex/WACC uplift applies to 2028-31 vintages only (x1.35/1.35/1.18/1.09); 2026-27 procured before the shock</t>
+          <t>funnel-released twin of every scenario except s05: parent overlays + gas guardrail minimum = residual capacity from 2031 (announced projects through 2030 kept), build-rate caps unchanged; base NOT released (user decision)</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Review #6: shock cancelled projects already under construction</t>
+          <t>review item 2 / funnel debate: forced 366 GW of new CCGT+OCGT contradict s14/s07/s12; s05 already releases from 2027</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>fel2026_s06_hormuz_49_2015_v6_v2</t>
+          <t>fel2026_sNN_&lt;name&gt;_open_49_2015_v6</t>
         </is>
       </c>
     </row>
@@ -1311,17 +1771,17 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>ITC restoration phased in: capex x0.90 (2029), x0.80 (2030), x0.70 (2031+); CCS via GasCCS/USA group cap 40 GW; mode-2 overlay now redundant (in base)</t>
+          <t>no change; results now report ITC (193 bEUR disc.), 45Q (24) and CO2 payments (322) -&gt; resource cost +166 bEUR</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Review #7: +130 GW solar spike in 2029</t>
+          <t>N3</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>fel2026_s14_decarb_49_2015_v6_v4</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1789,7 @@
       <c r="A9" s="9" t="inlineStr"/>
       <c r="B9" s="9" t="inlineStr"/>
       <c r="C9" s="9" t="inlineStr"/>
-      <c r="D9" s="9" t="n"/>
+      <c r="D9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1339,7 +1799,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>docs/proposals/scenario_plan_2026-09-18/RESULTS_wave2_2026-09-24.md; table s14_summary_wave2.csv</t>
+          <t>docs/proposals/scenario_plan_2026-09-18/RESULTS_wave3_2026-09-25.md; response docs/proposals/scenario_results/REVIEW_RESPONSE_wave2_2026-09-24.md</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr"/>
@@ -1351,6 +1811,207 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Wave 2 (2026-09-23/24): all 14 scenarios and the base rerun on one identical setup after the wave-1 review</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>change vs plan v3 / wave 1</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>reason (review item)</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>wave-2 run label</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Biogas co-firing mode (mode 2, Gas_Bio) disabled for all gas plants in the BASE data (OutputActivityRatio Power = 0); new base RegularParameters_NorthAmerica_v6e</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Review #1: mode 2 = unlimited zero-CO2 gas in the power-only data, understated 2030 CO2 by ~600 Mt in every v6 run</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_base_49_2015_v6e</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>rerun on the fixed base data; definitions otherwise unchanged</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>identical setup across the set</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_sNN_&lt;name&gt;_49_2015_v6_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>s03</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>crypto adder = growth above today's load: 0 TWh 2026, +10 TWh 2030, +20 TWh 2035/40 (was on from 2025)</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Review #3: crypto double-counted (already in the FEL base load)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s03_compute_49_2015_v6_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>s05</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>separate GasEngines window cap (min(base,1) GW/yr 2027-31) next to the GasPlants cap min(base,10) GW/yr 2027-31; engines NOT in GasPlants (base GasPlants 6/9/10 GW caps would collide)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Review #12: 2028 gas additions exceeded the cap via engines outside the subset</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s05_brakes_49_2015_v6_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>s06</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>capex/WACC uplift applies to 2028-31 vintages only (x1.35/1.35/1.18/1.09); 2026-27 procured before the shock</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Review #6: shock cancelled projects already under construction</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s06_hormuz_49_2015_v6_v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>s14</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>ITC restoration phased in: capex x0.90 (2029), x0.80 (2030), x0.70 (2031+); CCS via GasCCS/USA group cap 40 GW; mode-2 overlay now redundant (in base)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Review #7: +130 GW solar spike in 2029</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>fel2026_s14_decarb_49_2015_v6_v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr"/>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>results</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>docs/proposals/scenario_plan_2026-09-18/RESULTS_wave2_2026-09-24.md; table s14_summary_wave2.csv</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2433,7 +3094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9184,7 +9845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10109,7 +10770,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14612,7 +15273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15345,155 +16006,4 @@
   <autoFilter ref="A1:F37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Sensitivity (v6 set)</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>dc_high</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>DC US 2035/2040 = 2188/3585 TWh; funnel max raised with ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>dc_low</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>DC US 2035/2040 = 805/874 TWh; gas min floor 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>recession</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>GDP-recession FEL demand: DC 1048/1563, General -1..2 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>btm_lag</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>DC 1526/2163 (BTM lag -&gt; more grid load)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>economic</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>funnel widened after 2030 (min x0.75, max x1.5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>grid_high/grid_low</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>IC growth 2x budget / capped 0.75 %/yr</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>bess_optimistic/pessimistic</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Li-ion cost x0.4 by 2040 + 7 h / min blend x0.53</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>nuclear_announced (+ccgtrelax)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>+19.1 GW announced nuclear (large+SMR) by 2035 on top of the corridor, CCGT min relaxed</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>space_dc / disruptive / spacex</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>orbital compute REMOVES 5 / 13 / 27 % of US DC load by 2040 (1724/1585/1353 TWh)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>gas (NorthAmerica_gas)</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>explicit gas supply, pipelines, LNG exports, storage, deliverability caps; endogenous regional gas prices</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B11"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>